<commit_message>
Restructure reports: DayViol/MonthViol presets, XLSX evidence, remove PPTX
Major changes:
- New XML presets: Report A (Daily, DayViol marker) and Report B (Monthly,
  MonthViol marker) in src/presets/
- Flow definition: XPath now reads DayViol/MonthViol instead of ViolationMarker
- Evidence storage: XLSX files instead of CSV, with styled headers and
  color-coded status. Original XML archived to /Evidence Archive/XML Archive/
- Removed all PPTX template infrastructure (daily_run_template.pptx,
  PopulateTemplate action, Presentation_Link column)
- Replaced per-run presentations with single consolidated findings deck
  (generate_findings_presentation.py)
- Updated SharePoint schema: removed Presentation_Link, fixed column names
- Deleted old test runs (will be regenerated with new XML structure)
- Updated README, SharePoint guide, and tests README with new architecture
</commit_message>
<xml_diff>
--- a/tests/Email_Report_Schema (1).xlsx
+++ b/tests/Email_Report_Schema (1).xlsx
@@ -127,7 +127,7 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>ChatGPT</author>
+    <author>ISAAI</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
@@ -182,17 +182,12 @@
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>Link to Report A Excel evidence file</t>
+        <t>Link to Report A Excel evidence file (.xlsx)</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
       <text>
-        <t>Link to Report B Excel evidence file</t>
-      </text>
-    </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
-      <text>
-        <t>Link to generated PowerPoint deck</t>
+        <t>Link to Report B Excel evidence file (.xlsx)</t>
       </text>
     </comment>
   </commentList>
@@ -488,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -567,11 +562,6 @@
           <t>EvidenceB_Link</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Presentation_Link</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <dataValidations count="3">

</xml_diff>